<commit_message>
Entry Fee v5: Gate 3 close, Workbook B reconciliation, tie-out and cover note
Reconcile the report to the Model agent's tie-out: Exhibit 18b and the section 12 verdict
now print the Workbook B vertically-integrated figures (56,811 to first frontier model,
81,229 to first $1B) with the superseded pre-model bands stated; named ranges LB_01-LB_10;
Riot start assumption and the 8.135 composite stated in the text. Rebuilt and validated the
docx, re-rendered the PDF, updated the figure register and changelog. Added the Model agent's
final workbooks, sweep and cross-check scripts, tie-out.md, GATE3.md as PASS, and the final
cover note.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XNwUojzXk86a8Dfphw26Rp
</commit_message>
<xml_diff>
--- a/entry-fee/model/entry-fee-v5.xlsx
+++ b/entry-fee/model/entry-fee-v5.xlsx
@@ -24,22 +24,22 @@
     <sheet name="13_OutsideView" sheetId="14" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="LB01" vbProcedure="false">01_Data!$D$5</definedName>
-    <definedName function="false" hidden="false" name="LB02" vbProcedure="false">01_Data!$D$6</definedName>
-    <definedName function="false" hidden="false" name="LB03" vbProcedure="false">01_Data!$D$7</definedName>
-    <definedName function="false" hidden="false" name="LB04" vbProcedure="false">01_Data!$D$8</definedName>
-    <definedName function="false" hidden="false" name="LB05" vbProcedure="false">01_Data!$D$9</definedName>
-    <definedName function="false" hidden="false" name="LB05a" vbProcedure="false">01_Data!$D$9</definedName>
-    <definedName function="false" hidden="false" name="LB05b" vbProcedure="false">01_Data!$D$11</definedName>
-    <definedName function="false" hidden="false" name="LB06" vbProcedure="false">01_Data!$D$16</definedName>
-    <definedName function="false" hidden="false" name="LB06a" vbProcedure="false">01_Data!$D$16</definedName>
-    <definedName function="false" hidden="false" name="LB06b" vbProcedure="false">01_Data!$D$18</definedName>
-    <definedName function="false" hidden="false" name="LB07" vbProcedure="false">01_Data!$D$19</definedName>
-    <definedName function="false" hidden="false" name="LB07a" vbProcedure="false">01_Data!$D$19</definedName>
-    <definedName function="false" hidden="false" name="LB07b" vbProcedure="false">01_Data!$D$20</definedName>
-    <definedName function="false" hidden="false" name="LB08" vbProcedure="false">01_Data!$D$23</definedName>
-    <definedName function="false" hidden="false" name="LB09" vbProcedure="false">01_Data!$D$25</definedName>
-    <definedName function="false" hidden="false" name="LB10" vbProcedure="false">01_Data!$D$31</definedName>
+    <definedName function="false" hidden="false" name="LB_01" vbProcedure="false">01_Data!$D$5</definedName>
+    <definedName function="false" hidden="false" name="LB_02" vbProcedure="false">01_Data!$D$6</definedName>
+    <definedName function="false" hidden="false" name="LB_03" vbProcedure="false">01_Data!$D$7</definedName>
+    <definedName function="false" hidden="false" name="LB_04" vbProcedure="false">01_Data!$D$8</definedName>
+    <definedName function="false" hidden="false" name="LB_05" vbProcedure="false">01_Data!$D$9</definedName>
+    <definedName function="false" hidden="false" name="LB_05a" vbProcedure="false">01_Data!$D$9</definedName>
+    <definedName function="false" hidden="false" name="LB_05b" vbProcedure="false">01_Data!$D$11</definedName>
+    <definedName function="false" hidden="false" name="LB_06" vbProcedure="false">01_Data!$D$16</definedName>
+    <definedName function="false" hidden="false" name="LB_06a" vbProcedure="false">01_Data!$D$16</definedName>
+    <definedName function="false" hidden="false" name="LB_06b" vbProcedure="false">01_Data!$D$18</definedName>
+    <definedName function="false" hidden="false" name="LB_07" vbProcedure="false">01_Data!$D$19</definedName>
+    <definedName function="false" hidden="false" name="LB_07a" vbProcedure="false">01_Data!$D$19</definedName>
+    <definedName function="false" hidden="false" name="LB_07b" vbProcedure="false">01_Data!$D$20</definedName>
+    <definedName function="false" hidden="false" name="LB_08" vbProcedure="false">01_Data!$D$23</definedName>
+    <definedName function="false" hidden="false" name="LB_09" vbProcedure="false">01_Data!$D$25</definedName>
+    <definedName function="false" hidden="false" name="LB_10" vbProcedure="false">01_Data!$D$31</definedName>
     <definedName function="false" hidden="false" name="SW_15B_FACILITY" vbProcedure="false">12_Conflicts!$C$14</definedName>
     <definedName function="false" hidden="false" name="SW_A_2026_LOSS" vbProcedure="false">12_Conflicts!$C$10</definedName>
     <definedName function="false" hidden="false" name="SW_A_FY24_NI" vbProcedure="false">12_Conflicts!$C$9</definedName>
@@ -16188,7 +16188,7 @@
         <v>250,000 incremental commitment: could-not-verify (register); T1 facts: revenue share through 2030 at the same % subject to a cap; non-exclusive IP to 2032; any cloud</v>
       </c>
       <c r="C26" s="31" t="n">
-        <f aca="false">LB08</f>
+        <f aca="false">LB_08</f>
         <v>24100</v>
       </c>
       <c r="D26" s="31" t="str">
@@ -16596,7 +16596,7 @@
         <v>2770</v>
       </c>
       <c r="E40" s="31" t="n">
-        <f aca="false">LB08+LB07a+01_Data!$D$252+01_Data!$D$160</f>
+        <f aca="false">LB_08+LB_07a+01_Data!$D$252+01_Data!$D$160</f>
         <v>78800</v>
       </c>
     </row>
@@ -16917,7 +16917,7 @@
         <v>2825</v>
       </c>
       <c r="D56" s="31" t="n">
-        <f aca="false">LB07b</f>
+        <f aca="false">LB_07b</f>
         <v>750000</v>
       </c>
       <c r="E56" s="2" t="s">
@@ -16972,7 +16972,7 @@
         <v>2835</v>
       </c>
       <c r="D58" s="31" t="n">
-        <f aca="false">LB07a</f>
+        <f aca="false">LB_07a</f>
         <v>50000</v>
       </c>
       <c r="E58" s="2" t="s">
@@ -17608,7 +17608,7 @@
         <v>65800</v>
       </c>
       <c r="I82" s="31" t="n">
-        <f aca="false">LB10*(1-01_Data!$D$65)+01_Data!$D$68</f>
+        <f aca="false">LB_10*(1-01_Data!$D$65)+01_Data!$D$68</f>
         <v>65700</v>
       </c>
       <c r="J82" s="65" t="s">
@@ -20186,7 +20186,7 @@
         <v>120500</v>
       </c>
       <c r="I118" s="31" t="n">
-        <f aca="false">LB08</f>
+        <f aca="false">LB_08</f>
         <v>24100</v>
       </c>
       <c r="J118" s="2" t="s">
@@ -23672,7 +23672,7 @@
         <v>3461</v>
       </c>
       <c r="F11" s="57" t="str">
-        <f aca="false">"Q2 adjusted margin ~"&amp;TEXT(LB05b/01_Data!$D$12,"0.0%")</f>
+        <f aca="false">"Q2 adjusted margin ~"&amp;TEXT(LB_05b/01_Data!$D$12,"0.0%")</f>
         <v>Q2 adjusted margin ~5.1%</v>
       </c>
       <c r="G11" s="2" t="s">
@@ -24035,7 +24035,7 @@
         <v>PASS</v>
       </c>
       <c r="F29" s="31" t="n">
-        <f aca="false">LB10</f>
+        <f aca="false">LB_10</f>
         <v>190000</v>
       </c>
       <c r="G29" s="31" t="n">
@@ -39543,7 +39543,7 @@
         <v>320</v>
       </c>
       <c r="E9" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -39615,7 +39615,7 @@
         <v>330</v>
       </c>
       <c r="E13" s="31" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -39708,7 +39708,7 @@
         <v>351</v>
       </c>
       <c r="E19" s="31" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -39763,7 +39763,7 @@
         <v>351</v>
       </c>
       <c r="E22" s="31" t="n">
-        <f aca="false">LB06a</f>
+        <f aca="false">LB_06a</f>
         <v>6700</v>
       </c>
       <c r="F22" s="2" t="s">
@@ -39995,7 +39995,7 @@
         <v>2025</v>
       </c>
       <c r="D35" s="11" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -40032,7 +40032,7 @@
         <v>2025</v>
       </c>
       <c r="D37" s="11" t="n">
-        <f aca="false">LB01*(1-SW_HAIRCUT)</f>
+        <f aca="false">LB_01*(1-SW_HAIRCUT)</f>
         <v>39162.5</v>
       </c>
       <c r="E37" s="62" t="n">
@@ -40051,7 +40051,7 @@
         <v>2025</v>
       </c>
       <c r="D38" s="11" t="n">
-        <f aca="false">LB01*(1-01_Data!$D$36)</f>
+        <f aca="false">LB_01*(1-01_Data!$D$36)</f>
         <v>39162.5</v>
       </c>
       <c r="E38" s="62" t="n">
@@ -40074,7 +40074,7 @@
         <v>2025</v>
       </c>
       <c r="D39" s="11" t="n">
-        <f aca="false">LB01*(1-01_Data!$D$37)</f>
+        <f aca="false">LB_01*(1-01_Data!$D$37)</f>
         <v>47450</v>
       </c>
       <c r="E39" s="62" t="n">
@@ -40112,7 +40112,7 @@
         <v>2025</v>
       </c>
       <c r="D41" s="11" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="E41" s="2" t="s">
@@ -40149,7 +40149,7 @@
         <v>2025</v>
       </c>
       <c r="D43" s="11" t="n">
-        <f aca="false">IF(SW_OAI_BASIS="NET",LB02,LB02*(1-01_Data!$D$38))</f>
+        <f aca="false">IF(SW_OAI_BASIS="NET",LB_02,LB_02*(1-01_Data!$D$38))</f>
         <v>40000</v>
       </c>
       <c r="E43" s="62" t="n">
@@ -40168,7 +40168,7 @@
         <v>2025</v>
       </c>
       <c r="D44" s="11" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="E44" s="2" t="s">
@@ -40186,7 +40186,7 @@
         <v>2025</v>
       </c>
       <c r="D45" s="11" t="n">
-        <f aca="false">LB02*(1-01_Data!$D$38)</f>
+        <f aca="false">LB_02*(1-01_Data!$D$38)</f>
         <v>32000</v>
       </c>
       <c r="E45" s="13" t="n">
@@ -40208,7 +40208,7 @@
         <v>2025</v>
       </c>
       <c r="D46" s="11" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="E46" s="2" t="s">
@@ -40226,7 +40226,7 @@
         <v>2025</v>
       </c>
       <c r="D47" s="11" t="n">
-        <f aca="false">LB05a*(1-01_Data!$D$36)</f>
+        <f aca="false">LB_05a*(1-01_Data!$D$36)</f>
         <v>6989</v>
       </c>
       <c r="E47" s="62" t="n">
@@ -40245,7 +40245,7 @@
         <v>2025</v>
       </c>
       <c r="D48" s="11" t="n">
-        <f aca="false">LB05a*(1-01_Data!$D$37)</f>
+        <f aca="false">LB_05a*(1-01_Data!$D$37)</f>
         <v>8468</v>
       </c>
       <c r="E48" s="62" t="n">
@@ -40264,7 +40264,7 @@
         <v>2025</v>
       </c>
       <c r="D49" s="11" t="n">
-        <f aca="false">LB06a</f>
+        <f aca="false">LB_06a</f>
         <v>6700</v>
       </c>
       <c r="E49" s="2" t="s">
@@ -40374,7 +40374,7 @@
         <v>2061</v>
       </c>
       <c r="D54" s="31" t="n">
-        <f aca="false">LB01/00_Assumptions!$D$90</f>
+        <f aca="false">LB_01/00_Assumptions!$D$90</f>
         <v>5416.66666666667</v>
       </c>
       <c r="E54" s="32" t="n">
@@ -40406,7 +40406,7 @@
         <v>25250</v>
       </c>
       <c r="L54" s="31" t="n">
-        <f aca="false">01_Data!$D$13+LB05a</f>
+        <f aca="false">01_Data!$D$13+LB_05a</f>
         <v>16330</v>
       </c>
       <c r="M54" s="64" t="n">
@@ -40430,7 +40430,7 @@
         <v>2063</v>
       </c>
       <c r="D55" s="31" t="n">
-        <f aca="false">LB01/00_Assumptions!$D$90</f>
+        <f aca="false">LB_01/00_Assumptions!$D$90</f>
         <v>5416.66666666667</v>
       </c>
       <c r="E55" s="32" t="n">
@@ -40462,7 +40462,7 @@
         <v>23250</v>
       </c>
       <c r="L55" s="31" t="n">
-        <f aca="false">01_Data!$D$13+LB05a</f>
+        <f aca="false">01_Data!$D$13+LB_05a</f>
         <v>16330</v>
       </c>
       <c r="M55" s="64" t="n">
@@ -40490,7 +40490,7 @@
         <v>2063</v>
       </c>
       <c r="D56" s="31" t="n">
-        <f aca="false">LB01/00_Assumptions!$D$90</f>
+        <f aca="false">LB_01/00_Assumptions!$D$90</f>
         <v>5416.66666666667</v>
       </c>
       <c r="E56" s="32" t="n">
@@ -40522,7 +40522,7 @@
         <v>27250</v>
       </c>
       <c r="L56" s="31" t="n">
-        <f aca="false">01_Data!$D$13+LB05a</f>
+        <f aca="false">01_Data!$D$13+LB_05a</f>
         <v>16330</v>
       </c>
       <c r="M56" s="64" t="n">
@@ -40543,14 +40543,14 @@
         <v>2065</v>
       </c>
       <c r="B57" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>2066</v>
       </c>
       <c r="D57" s="31" t="n">
-        <f aca="false">LB01/00_Assumptions!$D$90</f>
+        <f aca="false">LB_01/00_Assumptions!$D$90</f>
         <v>5416.66666666667</v>
       </c>
       <c r="E57" s="32" t="n">
@@ -40582,7 +40582,7 @@
         <v>16250</v>
       </c>
       <c r="L57" s="31" t="n">
-        <f aca="false">01_Data!$D$13+LB05a</f>
+        <f aca="false">01_Data!$D$13+LB_05a</f>
         <v>16330</v>
       </c>
       <c r="M57" s="64" t="n">
@@ -40708,7 +40708,7 @@
         <v>2074</v>
       </c>
       <c r="D64" s="31" t="n">
-        <f aca="false">LB02/00_Assumptions!$D$90</f>
+        <f aca="false">LB_02/00_Assumptions!$D$90</f>
         <v>3333.33333333333</v>
       </c>
       <c r="E64" s="32" t="n">
@@ -40740,7 +40740,7 @@
         <v>14685.3666666667</v>
       </c>
       <c r="L64" s="31" t="n">
-        <f aca="false">01_Data!$D$15+LB06a</f>
+        <f aca="false">01_Data!$D$15+LB_06a</f>
         <v>12400</v>
       </c>
       <c r="M64" s="64" t="n">
@@ -40760,7 +40760,7 @@
         <v>2074</v>
       </c>
       <c r="D65" s="31" t="n">
-        <f aca="false">LB02/00_Assumptions!$D$90</f>
+        <f aca="false">LB_02/00_Assumptions!$D$90</f>
         <v>3333.33333333333</v>
       </c>
       <c r="E65" s="32" t="n">
@@ -40792,7 +40792,7 @@
         <v>10000</v>
       </c>
       <c r="L65" s="31" t="n">
-        <f aca="false">01_Data!$D$15+LB06a</f>
+        <f aca="false">01_Data!$D$15+LB_06a</f>
         <v>12400</v>
       </c>
       <c r="M65" s="64" t="n">
@@ -40816,7 +40816,7 @@
         <v>2074</v>
       </c>
       <c r="D66" s="31" t="n">
-        <f aca="false">LB02/00_Assumptions!$D$90</f>
+        <f aca="false">LB_02/00_Assumptions!$D$90</f>
         <v>3333.33333333333</v>
       </c>
       <c r="E66" s="32" t="n">
@@ -40848,7 +40848,7 @@
         <v>14685.3666666667</v>
       </c>
       <c r="L66" s="31" t="n">
-        <f aca="false">01_Data!$D$15+LB06a</f>
+        <f aca="false">01_Data!$D$15+LB_06a</f>
         <v>12400</v>
       </c>
       <c r="M66" s="64" t="n">
@@ -40872,7 +40872,7 @@
         <v>2074</v>
       </c>
       <c r="D67" s="31" t="n">
-        <f aca="false">LB02/00_Assumptions!$D$90</f>
+        <f aca="false">LB_02/00_Assumptions!$D$90</f>
         <v>3333.33333333333</v>
       </c>
       <c r="E67" s="32" t="n">
@@ -40904,7 +40904,7 @@
         <v>20966.4</v>
       </c>
       <c r="L67" s="31" t="n">
-        <f aca="false">01_Data!$D$15+LB06a</f>
+        <f aca="false">01_Data!$D$15+LB_06a</f>
         <v>12400</v>
       </c>
       <c r="M67" s="64" t="n">
@@ -42692,7 +42692,7 @@
         <v>2163</v>
       </c>
       <c r="D49" s="31" t="n">
-        <f aca="false">LB07a</f>
+        <f aca="false">LB_07a</f>
         <v>50000</v>
       </c>
       <c r="E49" s="31" t="n">
@@ -42754,15 +42754,15 @@
         <v>2170</v>
       </c>
       <c r="D53" s="31" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="E53" s="31" t="n">
-        <f aca="false">LB05a*(1-01_Data!$D$36)</f>
+        <f aca="false">LB_05a*(1-01_Data!$D$36)</f>
         <v>6989</v>
       </c>
       <c r="F53" s="31" t="n">
-        <f aca="false">LB05a*(1-01_Data!$D$37)</f>
+        <f aca="false">LB_05a*(1-01_Data!$D$37)</f>
         <v>8468</v>
       </c>
     </row>
@@ -42778,15 +42778,15 @@
         <v>3000</v>
       </c>
       <c r="D54" s="51" t="n">
-        <f aca="false">(LB05b+$C54)/D$53</f>
+        <f aca="false">(LB_05b+$C54)/D$53</f>
         <v>0.306810344827586</v>
       </c>
       <c r="E54" s="51" t="n">
-        <f aca="false">(LB05b+$C54)/E$53</f>
+        <f aca="false">(LB_05b+$C54)/E$53</f>
         <v>0.509228788095579</v>
       </c>
       <c r="F54" s="51" t="n">
-        <f aca="false">(LB05b+$C54)/F$53</f>
+        <f aca="false">(LB_05b+$C54)/F$53</f>
         <v>0.420288143599433</v>
       </c>
       <c r="G54" s="7" t="str">
@@ -42813,15 +42813,15 @@
         <v>4000</v>
       </c>
       <c r="D55" s="51" t="n">
-        <f aca="false">(LB05b+$C55)/D$53</f>
+        <f aca="false">(LB_05b+$C55)/D$53</f>
         <v>0.39301724137931</v>
       </c>
       <c r="E55" s="51" t="n">
-        <f aca="false">(LB05b+$C55)/E$53</f>
+        <f aca="false">(LB_05b+$C55)/E$53</f>
         <v>0.652310774073544</v>
       </c>
       <c r="F55" s="51" t="n">
-        <f aca="false">(LB05b+$C55)/F$53</f>
+        <f aca="false">(LB_05b+$C55)/F$53</f>
         <v>0.538379782711384</v>
       </c>
     </row>
@@ -42837,15 +42837,15 @@
         <v>5000</v>
       </c>
       <c r="D56" s="51" t="n">
-        <f aca="false">(LB05b+$C56)/D$53</f>
+        <f aca="false">(LB_05b+$C56)/D$53</f>
         <v>0.479224137931034</v>
       </c>
       <c r="E56" s="51" t="n">
-        <f aca="false">(LB05b+$C56)/E$53</f>
+        <f aca="false">(LB_05b+$C56)/E$53</f>
         <v>0.79539276005151</v>
       </c>
       <c r="F56" s="51" t="n">
-        <f aca="false">(LB05b+$C56)/F$53</f>
+        <f aca="false">(LB_05b+$C56)/F$53</f>
         <v>0.656471421823335</v>
       </c>
     </row>
@@ -42884,7 +42884,7 @@
         <v>2177</v>
       </c>
       <c r="D59" s="51" t="n">
-        <f aca="false">00_Assumptions!$D$15/LB05a</f>
+        <f aca="false">00_Assumptions!$D$15/LB_05a</f>
         <v>0.258620689655172</v>
       </c>
       <c r="E59" s="61" t="str">
@@ -43918,11 +43918,11 @@
         <v>2226</v>
       </c>
       <c r="D33" s="11" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="E33" s="11" t="n">
-        <f aca="false">LB06a</f>
+        <f aca="false">LB_06a</f>
         <v>6700</v>
       </c>
       <c r="F33" s="2" t="s">
@@ -43994,11 +43994,11 @@
         <v>2231</v>
       </c>
       <c r="D36" s="11" t="n">
-        <f aca="false">LB05b</f>
+        <f aca="false">LB_05b</f>
         <v>559</v>
       </c>
       <c r="E36" s="11" t="n">
-        <f aca="false">-LB06b</f>
+        <f aca="false">-LB_06b</f>
         <v>-12300</v>
       </c>
       <c r="F36" s="2" t="s">
@@ -44037,7 +44037,7 @@
         <v>2237</v>
       </c>
       <c r="D38" s="14" t="n">
-        <f aca="false">LB05b/01_Data!$D$12</f>
+        <f aca="false">LB_05b/01_Data!$D$12</f>
         <v>0.0512844036697248</v>
       </c>
       <c r="E38" s="67" t="n">
@@ -44045,7 +44045,7 @@
         <v>1.74193548387097</v>
       </c>
       <c r="F38" s="51" t="n">
-        <f aca="false">LB05b/LB05a</f>
+        <f aca="false">LB_05b/LB_05a</f>
         <v>0.0481896551724138</v>
       </c>
       <c r="G38" s="2" t="s">
@@ -44066,7 +44066,7 @@
         <v>511</v>
       </c>
       <c r="E39" s="14" t="n">
-        <f aca="false">LB06b/01_Data!$D$17-1</f>
+        <f aca="false">LB_06b/01_Data!$D$17-1</f>
         <v>0.32258064516129</v>
       </c>
       <c r="F39" s="2" t="s">
@@ -44088,7 +44088,7 @@
         <v>16230</v>
       </c>
       <c r="E40" s="11" t="n">
-        <f aca="false">-(01_Data!$D$17+LB06b)</f>
+        <f aca="false">-(01_Data!$D$17+LB_06b)</f>
         <v>-21600</v>
       </c>
       <c r="F40" s="2"/>
@@ -44483,8 +44483,8 @@
         <v>124254</v>
       </c>
       <c r="E15" s="7" t="str">
-        <f aca="false">IF(ABS(D15-LB03)&lt;00_Assumptions!$E$132,"ties to LB03 (124,254)","BROKEN")</f>
-        <v>ties to LB03 (124,254)</v>
+        <f aca="false">IF(ABS(D15-LB_03)&lt;00_Assumptions!$E$132,"ties to LB_03 (124,254)","BROKEN")</f>
+        <v>ties to LB_03 (124,254)</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>2273</v>
@@ -44494,8 +44494,8 @@
         <v>181216.5</v>
       </c>
       <c r="K15" s="7" t="str">
-        <f aca="false">IF(ABS(J15-LB04)&lt;00_Assumptions!$E$133,"ties to LB04 (181,216.5)","BROKEN")</f>
-        <v>ties to LB04 (181,216.5)</v>
+        <f aca="false">IF(ABS(J15-LB_04)&lt;00_Assumptions!$E$133,"ties to LB_04 (181,216.5)","BROKEN")</f>
+        <v>ties to LB_04 (181,216.5)</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -44525,7 +44525,7 @@
         <v>2278</v>
       </c>
       <c r="D17" s="11" t="n">
-        <f aca="false">LB03+D16</f>
+        <f aca="false">LB_03+D16</f>
         <v>126754</v>
       </c>
       <c r="E17" s="7" t="str">
@@ -44540,7 +44540,7 @@
         <v>2279</v>
       </c>
       <c r="J17" s="71" t="n">
-        <f aca="false">LB04+J16</f>
+        <f aca="false">LB_04+J16</f>
         <v>186436.5</v>
       </c>
       <c r="K17" s="7" t="str">
@@ -44596,7 +44596,7 @@
         <v>1100</v>
       </c>
       <c r="K19" s="62" t="n">
-        <f aca="false">J19/LB04</f>
+        <f aca="false">J19/LB_04</f>
         <v>0.0060700874368504</v>
       </c>
     </row>
@@ -44618,7 +44618,7 @@
         <v>2289</v>
       </c>
       <c r="J20" s="72" t="n">
-        <f aca="false">02_Revenue!$D$43/(LB04-J19)</f>
+        <f aca="false">02_Revenue!$D$43/(LB_04-J19)</f>
         <v>0.222078488089653</v>
       </c>
     </row>
@@ -44769,7 +44769,7 @@
         <v>28317.5</v>
       </c>
       <c r="E42" s="72" t="n">
-        <f aca="false">D42/LB03</f>
+        <f aca="false">D42/LB_03</f>
         <v>0.227900107843611</v>
       </c>
       <c r="F42" s="31" t="n">
@@ -44777,7 +44777,7 @@
         <v>25000</v>
       </c>
       <c r="G42" s="72" t="n">
-        <f aca="false">F42/LB04</f>
+        <f aca="false">F42/LB_04</f>
         <v>0.137956532655691</v>
       </c>
       <c r="H42" s="58" t="n">
@@ -44801,7 +44801,7 @@
         <v>2313</v>
       </c>
       <c r="B43" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C43" s="62" t="n">
@@ -44813,7 +44813,7 @@
         <v>39162.5</v>
       </c>
       <c r="E43" s="73" t="n">
-        <f aca="false">D43/LB03</f>
+        <f aca="false">D43/LB_03</f>
         <v>0.315181000209249</v>
       </c>
       <c r="F43" s="31" t="n">
@@ -44821,7 +44821,7 @@
         <v>40000</v>
       </c>
       <c r="G43" s="73" t="n">
-        <f aca="false">F43/LB04</f>
+        <f aca="false">F43/LB_04</f>
         <v>0.220730452249105</v>
       </c>
       <c r="H43" s="63" t="n">
@@ -44838,7 +44838,7 @@
         <v>2314</v>
       </c>
       <c r="B44" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C44" s="62" t="n">
@@ -44850,7 +44850,7 @@
         <v>39162.5</v>
       </c>
       <c r="E44" s="73" t="n">
-        <f aca="false">D44/LB03</f>
+        <f aca="false">D44/LB_03</f>
         <v>0.315181000209249</v>
       </c>
       <c r="F44" s="31" t="n">
@@ -44858,7 +44858,7 @@
         <v>40000</v>
       </c>
       <c r="G44" s="73" t="n">
-        <f aca="false">F44/LB04</f>
+        <f aca="false">F44/LB_04</f>
         <v>0.220730452249105</v>
       </c>
       <c r="H44" s="63" t="n">
@@ -44886,7 +44886,7 @@
         <v>2316</v>
       </c>
       <c r="B45" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C45" s="62" t="n">
@@ -44898,7 +44898,7 @@
         <v>47450</v>
       </c>
       <c r="E45" s="73" t="n">
-        <f aca="false">D45/LB03</f>
+        <f aca="false">D45/LB_03</f>
         <v>0.381879054195438</v>
       </c>
       <c r="F45" s="31" t="n">
@@ -44906,7 +44906,7 @@
         <v>40000</v>
       </c>
       <c r="G45" s="73" t="n">
-        <f aca="false">F45/LB04</f>
+        <f aca="false">F45/LB_04</f>
         <v>0.220730452249105</v>
       </c>
       <c r="H45" s="63" t="n">
@@ -44930,18 +44930,18 @@
         <v>2317</v>
       </c>
       <c r="B46" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C46" s="74" t="s">
         <v>511</v>
       </c>
       <c r="D46" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="E46" s="75" t="n">
-        <f aca="false">D46/LB03</f>
+        <f aca="false">D46/LB_03</f>
         <v>0.523121992048546</v>
       </c>
       <c r="F46" s="31" t="n">
@@ -44949,7 +44949,7 @@
         <v>40000</v>
       </c>
       <c r="G46" s="73" t="n">
-        <f aca="false">F46/LB04</f>
+        <f aca="false">F46/LB_04</f>
         <v>0.220730452249105</v>
       </c>
       <c r="H46" s="63" t="n">
@@ -44973,7 +44973,7 @@
         <v>2318</v>
       </c>
       <c r="B47" s="31" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="C47" s="62" t="n">
@@ -44985,7 +44985,7 @@
         <v>39162.5</v>
       </c>
       <c r="E47" s="73" t="n">
-        <f aca="false">D47/LB03</f>
+        <f aca="false">D47/LB_03</f>
         <v>0.315181000209249</v>
       </c>
       <c r="F47" s="31" t="n">
@@ -44993,7 +44993,7 @@
         <v>32000</v>
       </c>
       <c r="G47" s="73" t="n">
-        <f aca="false">F47/LB04</f>
+        <f aca="false">F47/LB_04</f>
         <v>0.176584361799284</v>
       </c>
       <c r="H47" s="63" t="n">
@@ -45154,7 +45154,7 @@
         <v>2332</v>
       </c>
       <c r="D58" s="31" t="n">
-        <f aca="false">AVERAGE(01_Data!$D$17,LB06b)*00_Assumptions!$F$90</f>
+        <f aca="false">AVERAGE(01_Data!$D$17,LB_06b)*00_Assumptions!$F$90</f>
         <v>43200</v>
       </c>
     </row>
@@ -45232,7 +45232,7 @@
         <v>2343</v>
       </c>
       <c r="D65" s="31" t="n">
-        <f aca="false">LB05b*00_Assumptions!$F$90</f>
+        <f aca="false">LB_05b*00_Assumptions!$F$90</f>
         <v>2236</v>
       </c>
     </row>
@@ -45425,7 +45425,7 @@
         <v>1554</v>
       </c>
       <c r="D7" s="79" t="n">
-        <f aca="false">D5/LB01</f>
+        <f aca="false">D5/LB_01</f>
         <v>14.8461538461538</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -46020,7 +46020,7 @@
         <v>2315</v>
       </c>
       <c r="C6" s="31" t="n">
-        <f aca="false">LB01*(1-A6)</f>
+        <f aca="false">LB_01*(1-A6)</f>
         <v>47450</v>
       </c>
       <c r="D6" s="79" t="n">
@@ -46028,7 +46028,7 @@
         <v>20.3371970495258</v>
       </c>
       <c r="E6" s="31" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="F6" s="79" t="n">
@@ -46040,7 +46040,7 @@
         <v>-0.0452020164541871</v>
       </c>
       <c r="H6" s="83" t="n">
-        <f aca="false">(C6/LB03)/(E6/LB04)</f>
+        <f aca="false">(C6/LB_03)/(E6/LB_04)</f>
         <v>1.73006964061519</v>
       </c>
       <c r="I6" s="7" t="str">
@@ -46061,7 +46061,7 @@
         <v>2315</v>
       </c>
       <c r="C7" s="31" t="n">
-        <f aca="false">LB01*(1-A7)</f>
+        <f aca="false">LB_01*(1-A7)</f>
         <v>43550</v>
       </c>
       <c r="D7" s="79" t="n">
@@ -46069,7 +46069,7 @@
         <v>22.158438576349</v>
       </c>
       <c r="E7" s="31" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="F7" s="79" t="n">
@@ -46081,7 +46081,7 @@
         <v>0.0403022805797666</v>
       </c>
       <c r="H7" s="83" t="n">
-        <f aca="false">(C7/LB03)/(E7/LB04)</f>
+        <f aca="false">(C7/LB_03)/(E7/LB_04)</f>
         <v>1.58787213590709</v>
       </c>
     </row>
@@ -46094,7 +46094,7 @@
         <v>2315</v>
       </c>
       <c r="C8" s="31" t="n">
-        <f aca="false">LB01*(1-A8)</f>
+        <f aca="false">LB_01*(1-A8)</f>
         <v>39162.5</v>
       </c>
       <c r="D8" s="79" t="n">
@@ -46102,7 +46102,7 @@
         <v>24.6409192467284</v>
       </c>
       <c r="E8" s="31" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="F8" s="79" t="n">
@@ -46114,7 +46114,7 @@
         <v>0.156850668860487</v>
       </c>
       <c r="H8" s="83" t="n">
-        <f aca="false">(C8/LB03)/(E8/LB04)</f>
+        <f aca="false">(C8/LB_03)/(E8/LB_04)</f>
         <v>1.42789994311048</v>
       </c>
       <c r="I8" s="7" t="str">
@@ -46135,7 +46135,7 @@
         <v>1979</v>
       </c>
       <c r="C10" s="31" t="n">
-        <f aca="false">LB01*(1-A10)</f>
+        <f aca="false">LB_01*(1-A10)</f>
         <v>47450</v>
       </c>
       <c r="D10" s="79" t="n">
@@ -46143,7 +46143,7 @@
         <v>20.3371970495258</v>
       </c>
       <c r="E10" s="31" t="n">
-        <f aca="false">LB02*(1-01_Data!$D$38)</f>
+        <f aca="false">LB_02*(1-01_Data!$D$38)</f>
         <v>32000</v>
       </c>
       <c r="F10" s="79" t="n">
@@ -46155,7 +46155,7 @@
         <v>-0.23616161316335</v>
       </c>
       <c r="H10" s="83" t="n">
-        <f aca="false">(C10/LB03)/(E10/LB04)</f>
+        <f aca="false">(C10/LB_03)/(E10/LB_04)</f>
         <v>2.16258705076899</v>
       </c>
     </row>
@@ -46168,7 +46168,7 @@
         <v>1979</v>
       </c>
       <c r="C11" s="31" t="n">
-        <f aca="false">LB01*(1-A11)</f>
+        <f aca="false">LB_01*(1-A11)</f>
         <v>43550</v>
       </c>
       <c r="D11" s="79" t="n">
@@ -46176,7 +46176,7 @@
         <v>22.158438576349</v>
       </c>
       <c r="E11" s="31" t="n">
-        <f aca="false">LB02*(1-01_Data!$D$38)</f>
+        <f aca="false">LB_02*(1-01_Data!$D$38)</f>
         <v>32000</v>
       </c>
       <c r="F11" s="79" t="n">
@@ -46188,7 +46188,7 @@
         <v>-0.167758175536187</v>
       </c>
       <c r="H11" s="83" t="n">
-        <f aca="false">(C11/LB03)/(E11/LB04)</f>
+        <f aca="false">(C11/LB_03)/(E11/LB_04)</f>
         <v>1.98484016988387</v>
       </c>
     </row>
@@ -46201,7 +46201,7 @@
         <v>1979</v>
       </c>
       <c r="C12" s="31" t="n">
-        <f aca="false">LB01*(1-A12)</f>
+        <f aca="false">LB_01*(1-A12)</f>
         <v>39162.5</v>
       </c>
       <c r="D12" s="79" t="n">
@@ -46209,7 +46209,7 @@
         <v>24.6409192467284</v>
       </c>
       <c r="E12" s="31" t="n">
-        <f aca="false">LB02*(1-01_Data!$D$38)</f>
+        <f aca="false">LB_02*(1-01_Data!$D$38)</f>
         <v>32000</v>
       </c>
       <c r="F12" s="79" t="n">
@@ -46221,7 +46221,7 @@
         <v>-0.0745194649116103</v>
       </c>
       <c r="H12" s="83" t="n">
-        <f aca="false">(C12/LB03)/(E12/LB04)</f>
+        <f aca="false">(C12/LB_03)/(E12/LB_04)</f>
         <v>1.7848749288881</v>
       </c>
       <c r="I12" s="7" t="str">
@@ -46645,15 +46645,15 @@
         <v>0.4</v>
       </c>
       <c r="B46" s="31" t="n">
-        <f aca="false">$E46-(B$45-LB07a)*$H$46-$G$46*$E46</f>
+        <f aca="false">$E46-(B$45-LB_07a)*$H$46-$G$46*$E46</f>
         <v>-89994.241456</v>
       </c>
       <c r="C46" s="31" t="n">
-        <f aca="false">$E46-(C$45-LB07a)*$H$46-$G$46*$E46</f>
+        <f aca="false">$E46-(C$45-LB_07a)*$H$46-$G$46*$E46</f>
         <v>-142494.241456</v>
       </c>
       <c r="D46" s="31" t="n">
-        <f aca="false">$E46-(D$45-LB07a)*$H$46-$G$46*$E46</f>
+        <f aca="false">$E46-(D$45-LB_07a)*$H$46-$G$46*$E46</f>
         <v>-194994.241456</v>
       </c>
       <c r="E46" s="31" t="n">
@@ -46679,15 +46679,15 @@
         <v>0.7</v>
       </c>
       <c r="B47" s="31" t="n">
-        <f aca="false">$E47-(B$45-LB07a)*$H$46-$G$46*$E47</f>
+        <f aca="false">$E47-(B$45-LB_07a)*$H$46-$G$46*$E47</f>
         <v>30359.835989</v>
       </c>
       <c r="C47" s="31" t="n">
-        <f aca="false">$E47-(C$45-LB07a)*$H$46-$G$46*$E47</f>
+        <f aca="false">$E47-(C$45-LB_07a)*$H$46-$G$46*$E47</f>
         <v>-22140.1640109999</v>
       </c>
       <c r="D47" s="31" t="n">
-        <f aca="false">$E47-(D$45-LB07a)*$H$46-$G$46*$E47</f>
+        <f aca="false">$E47-(D$45-LB_07a)*$H$46-$G$46*$E47</f>
         <v>-74640.164011</v>
       </c>
       <c r="E47" s="31" t="n">
@@ -46701,15 +46701,15 @@
         <v>1</v>
       </c>
       <c r="B48" s="31" t="n">
-        <f aca="false">$E48-(B$45-LB07a)*$H$46-$G$46*$E48</f>
+        <f aca="false">$E48-(B$45-LB_07a)*$H$46-$G$46*$E48</f>
         <v>234429.44</v>
       </c>
       <c r="C48" s="31" t="n">
-        <f aca="false">$E48-(C$45-LB07a)*$H$46-$G$46*$E48</f>
+        <f aca="false">$E48-(C$45-LB_07a)*$H$46-$G$46*$E48</f>
         <v>181929.44</v>
       </c>
       <c r="D48" s="31" t="n">
-        <f aca="false">$E48-(D$45-LB07a)*$H$46-$G$46*$E48</f>
+        <f aca="false">$E48-(D$45-LB_07a)*$H$46-$G$46*$E48</f>
         <v>129429.44</v>
       </c>
       <c r="E48" s="31" t="n">
@@ -46722,15 +46722,15 @@
         <v>2416</v>
       </c>
       <c r="B50" s="31" t="n">
-        <f aca="false">(B45-LB07a)*$H$46</f>
+        <f aca="false">(B45-LB_07a)*$H$46</f>
         <v>192500</v>
       </c>
       <c r="C50" s="31" t="n">
-        <f aca="false">(C45-LB07a)*$H$46</f>
+        <f aca="false">(C45-LB_07a)*$H$46</f>
         <v>245000</v>
       </c>
       <c r="D50" s="31" t="n">
-        <f aca="false">(D45-LB07a)*$H$46</f>
+        <f aca="false">(D45-LB_07a)*$H$46</f>
         <v>297500</v>
       </c>
     </row>
@@ -46888,14 +46888,14 @@
         <v>18</v>
       </c>
       <c r="C4" s="11" t="n">
-        <f aca="false">LB03</f>
+        <f aca="false">LB_03</f>
         <v>124254</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>2431</v>
       </c>
       <c r="E4" s="11" t="n">
-        <f aca="false">LB04</f>
+        <f aca="false">LB_04</f>
         <v>181216.5</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -46916,14 +46916,14 @@
         <v>14</v>
       </c>
       <c r="C5" s="11" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>2436</v>
       </c>
       <c r="E5" s="11" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="F5" s="57" t="str">
@@ -46975,14 +46975,14 @@
         <v>18</v>
       </c>
       <c r="C7" s="11" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>2443</v>
       </c>
       <c r="E7" s="11" t="n">
-        <f aca="false">LB06a</f>
+        <f aca="false">LB_06a</f>
         <v>6700</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -47003,14 +47003,14 @@
         <v>18</v>
       </c>
       <c r="C8" s="11" t="n">
-        <f aca="false">LB05b</f>
+        <f aca="false">LB_05b</f>
         <v>559</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>2448</v>
       </c>
       <c r="E8" s="11" t="n">
-        <f aca="false">-LB06b</f>
+        <f aca="false">-LB_06b</f>
         <v>-12300</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -47246,7 +47246,7 @@
         <v>2480</v>
       </c>
       <c r="C18" s="11" t="n">
-        <f aca="false">LB01</f>
+        <f aca="false">LB_01</f>
         <v>65000</v>
       </c>
       <c r="D18" s="2" t="s">
@@ -47273,7 +47273,7 @@
         <v>2483</v>
       </c>
       <c r="C19" s="11" t="n">
-        <f aca="false">LB02</f>
+        <f aca="false">LB_02</f>
         <v>40000</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -47300,7 +47300,7 @@
         <v>2486</v>
       </c>
       <c r="C20" s="11" t="n">
-        <f aca="false">LB03</f>
+        <f aca="false">LB_03</f>
         <v>124254</v>
       </c>
       <c r="D20" s="2" t="s">
@@ -47327,7 +47327,7 @@
         <v>2490</v>
       </c>
       <c r="C21" s="11" t="n">
-        <f aca="false">LB04</f>
+        <f aca="false">LB_04</f>
         <v>181216.5</v>
       </c>
       <c r="D21" s="2" t="s">
@@ -47354,7 +47354,7 @@
         <v>2493</v>
       </c>
       <c r="C22" s="11" t="n">
-        <f aca="false">LB05a</f>
+        <f aca="false">LB_05a</f>
         <v>11600</v>
       </c>
       <c r="D22" s="2" t="s">
@@ -47381,7 +47381,7 @@
         <v>2498</v>
       </c>
       <c r="C23" s="11" t="n">
-        <f aca="false">LB06a</f>
+        <f aca="false">LB_06a</f>
         <v>6700</v>
       </c>
       <c r="D23" s="2" t="s">
@@ -47408,7 +47408,7 @@
         <v>2501</v>
       </c>
       <c r="C24" s="11" t="n">
-        <f aca="false">LB07a</f>
+        <f aca="false">LB_07a</f>
         <v>50000</v>
       </c>
       <c r="D24" s="2" t="s">
@@ -47435,7 +47435,7 @@
         <v>2506</v>
       </c>
       <c r="C25" s="11" t="n">
-        <f aca="false">LB08</f>
+        <f aca="false">LB_08</f>
         <v>24100</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -47462,7 +47462,7 @@
         <v>2509</v>
       </c>
       <c r="C26" s="19" t="n">
-        <f aca="false">LB09</f>
+        <f aca="false">LB_09</f>
         <v>8</v>
       </c>
       <c r="D26" s="2" t="s">
@@ -47489,7 +47489,7 @@
         <v>2512</v>
       </c>
       <c r="C27" s="11" t="n">
-        <f aca="false">LB10</f>
+        <f aca="false">LB_10</f>
         <v>190000</v>
       </c>
       <c r="D27" s="2" t="s">
@@ -47513,26 +47513,26 @@
         <v>2514</v>
       </c>
       <c r="C28" s="11" t="n">
-        <f aca="false">LB05b</f>
+        <f aca="false">LB_05b</f>
         <v>559</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>2515</v>
       </c>
       <c r="E28" s="11" t="n">
-        <f aca="false">LB06b</f>
+        <f aca="false">LB_06b</f>
         <v>12300</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>2516</v>
       </c>
       <c r="G28" s="11" t="n">
-        <f aca="false">LB07b</f>
+        <f aca="false">LB_07b</f>
         <v>750000</v>
       </c>
       <c r="H28" s="57" t="str">
-        <f aca="false">"LB10 high = "&amp;TEXT(01_Data!$D$32,"#,##0")&amp;"; RVG = "&amp;TEXT(01_Data!$D$27,"#,##0")</f>
-        <v>LB10 high = 200,000; RVG = 105,000</v>
+        <f aca="false">"LB_10 high = "&amp;TEXT(01_Data!$D$32,"#,##0")&amp;"; RVG = "&amp;TEXT(01_Data!$D$27,"#,##0")</f>
+        <v>LB_10 high = 200,000; RVG = 105,000</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>